<commit_message>
Redefine computational error: allow 5% tolerance for LLM computation result, update corresponding v2 annotation files and few-shot examples
</commit_message>
<xml_diff>
--- a/error_analysis/Cohen's_kappa_result.xlsx
+++ b/error_analysis/Cohen's_kappa_result.xlsx
@@ -766,30 +766,30 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G7" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>0 / 50</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n">
         <v>1</v>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>4 / 50</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>0.822</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -865,26 +865,26 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H10" s="17" t="inlineStr"/>
       <c r="I10" s="18" t="n">
-        <v>0.721</v>
+        <v>0.751</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">

</xml_diff>